<commit_message>
Add Puerto Vallarta property images and update Santiago xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/imagenes/Santiago Nuevo Leon/1/Formato Santiago.xlsx
+++ b/backend/imagenes/Santiago Nuevo Leon/1/Formato Santiago.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Ciudad</t>
   </si>
@@ -62,6 +62,12 @@
   </si>
   <si>
     <t>si</t>
+  </si>
+  <si>
+    <t>Misión de Sta. Inés 36, Las Misiones, 67302 Santiago, N.L.</t>
+  </si>
+  <si>
+    <t>alberca,jacuzzi,gym,area de juegos infantiles,terraza,calefaccion,cine,AC</t>
   </si>
 </sst>
 </file>
@@ -392,6 +398,41 @@
         <v>16</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="1">
+        <v>65000.0</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="F3" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1350.0</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>